<commit_message>
change time of calendar
</commit_message>
<xml_diff>
--- a/python/calendar.xlsx
+++ b/python/calendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\c0a230775e\code\quasar\gurisuro-reservation\python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2432A3-B542-4E83-B6E7-E171F0CA82F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A45ECE-93AA-4B1A-A56B-D71E50383E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>日</t>
     <rPh sb="0" eb="1">
@@ -56,10 +56,6 @@
     <t>土</t>
   </si>
   <si>
-    <t>23/30</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t xml:space="preserve">12
 </t>
     <phoneticPr fontId="1"/>
@@ -89,21 +85,33 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>17
+フリー運行
+15:00-16:00</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>19
+フリー運行
+15:30-16:30</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>23/30
+フリー運行
+16:30-17:30</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>26
 フリー運行
-16:00-17:00</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>17
-フリー運行
-15:00-16:00</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>19
-フリー運行
-15:30-16:30</t>
+16:30-17:30</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>27
+フリー運行
+17:30-18:30</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -503,13 +511,13 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" s="2">
         <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" s="2">
         <v>6</v>
@@ -526,13 +534,13 @@
         <v>9</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="2">
         <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" s="2">
         <v>13</v>
@@ -549,13 +557,13 @@
         <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2">
         <v>18</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F6" s="2">
         <v>20</v>
@@ -568,20 +576,20 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="55" customHeight="1">
-      <c r="B7" s="2" t="s">
-        <v>7</v>
+      <c r="B7" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7" s="2">
         <v>25</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="2">
-        <v>27</v>
+        <v>15</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="G7" s="2">
         <v>28</v>

</xml_diff>